<commit_message>
Updated Excel valuation model
</commit_message>
<xml_diff>
--- a/SOFI_DCF_Model.xlsx
+++ b/SOFI_DCF_Model.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Steve\OneDrive\Desktop\Excel Projects\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Steve\OneDrive\Desktop\Excel Projects\sofi-valuation-model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F911992B-80D2-4CBD-810E-F6C47D15ABE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68669F3B-4F17-42CE-AB4F-C92B837666A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="90">
   <si>
     <t>Assumption</t>
   </si>
@@ -547,7 +547,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -645,7 +645,6 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="8" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1650,7 +1649,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B0EA69A-16BD-4699-B50A-83E8D9E94131}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.453125" customWidth="1"/>
@@ -1667,227 +1666,222 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>21</v>
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>28</v>
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="14">
+        <f>Historicals!E3</f>
+        <v>3613354</v>
+      </c>
+      <c r="C3" s="14">
+        <f>B3*(1+Assumptions!B2)</f>
+        <v>4336024.8</v>
+      </c>
+      <c r="D3" s="14">
+        <f>C3*(1+Assumptions!C2)</f>
+        <v>5116509.2639999995</v>
+      </c>
+      <c r="E3" s="14">
+        <f>D3*(1+Assumptions!D2)</f>
+        <v>5935150.7462399993</v>
+      </c>
+      <c r="F3" s="14">
+        <f>E3*(1+Assumptions!E2)</f>
+        <v>6766071.8507136004</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="B4" s="14">
-        <f>Historicals!E3</f>
-        <v>3613354</v>
+        <f>Historicals!E4</f>
+        <v>1100000</v>
       </c>
       <c r="C4" s="14">
-        <f>B4*(1+Assumptions!B2)</f>
-        <v>4336024.8</v>
+        <f>C3*Assumptions!B3</f>
+        <v>1344167.6879999998</v>
       </c>
       <c r="D4" s="14">
-        <f>C4*(1+Assumptions!C2)</f>
-        <v>5116509.2639999995</v>
+        <f>D3*Assumptions!C3</f>
+        <v>1637282.9644799998</v>
       </c>
       <c r="E4" s="14">
-        <f>D4*(1+Assumptions!D2)</f>
-        <v>5935150.7462399993</v>
+        <f>E3*Assumptions!D3</f>
+        <v>1958599.7462591999</v>
       </c>
       <c r="F4" s="14">
-        <f>E4*(1+Assumptions!E2)</f>
-        <v>6766071.8507136004</v>
+        <f>F3*Assumptions!E3</f>
+        <v>2300464.4292426244</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B5" s="14">
-        <f>Historicals!E4</f>
-        <v>1100000</v>
+        <f>Historicals!E5</f>
+        <v>481320</v>
       </c>
       <c r="C5" s="14">
-        <f>C4*Assumptions!B3</f>
-        <v>1344167.6879999998</v>
+        <f>C3*Assumptions!B7</f>
+        <v>607043.47200000007</v>
       </c>
       <c r="D5" s="14">
-        <f>D4*Assumptions!C3</f>
-        <v>1637282.9644799998</v>
+        <f>D3*Assumptions!C7</f>
+        <v>767476.38959999988</v>
       </c>
       <c r="E5" s="14">
-        <f>E4*Assumptions!D3</f>
-        <v>1958599.7462591999</v>
+        <f>E3*Assumptions!D7</f>
+        <v>949624.11939839995</v>
       </c>
       <c r="F5" s="14">
-        <f>F4*Assumptions!E3</f>
-        <v>2300464.4292426244</v>
+        <f>F3*Assumptions!E7</f>
+        <v>1082571.496114176</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="B6" s="14">
-        <f>Historicals!E5</f>
-        <v>481320</v>
+        <f>Historicals!E7</f>
+        <v>242444</v>
       </c>
       <c r="C6" s="14">
-        <f>C4*Assumptions!B7</f>
-        <v>607043.47200000007</v>
+        <f>C3*Assumptions!B5</f>
+        <v>216801.24</v>
       </c>
       <c r="D6" s="14">
-        <f>D4*Assumptions!C7</f>
-        <v>767476.38959999988</v>
+        <f>D3*Assumptions!C5</f>
+        <v>255825.4632</v>
       </c>
       <c r="E6" s="14">
-        <f>E4*Assumptions!D7</f>
-        <v>949624.11939839995</v>
+        <f>E3*Assumptions!D5</f>
+        <v>296757.537312</v>
       </c>
       <c r="F6" s="14">
-        <f>F4*Assumptions!E7</f>
-        <v>1082571.496114176</v>
+        <f>F3*Assumptions!E5</f>
+        <v>338303.59253568004</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B7" s="14">
-        <f>Historicals!E7</f>
-        <v>242444</v>
+        <f>Historicals!E10</f>
+        <v>38037063</v>
       </c>
       <c r="C7" s="14">
-        <f>C4*Assumptions!B5</f>
-        <v>216801.24</v>
+        <f>B7*(1+Assumptions!B8)</f>
+        <v>47546328.75</v>
       </c>
       <c r="D7" s="14">
-        <f>D4*Assumptions!C5</f>
-        <v>255825.4632</v>
+        <f>C7*(1+Assumptions!C8)</f>
+        <v>58006521.074999996</v>
       </c>
       <c r="E7" s="14">
-        <f>E4*Assumptions!D5</f>
-        <v>296757.537312</v>
+        <f>D7*(1+Assumptions!D8)</f>
+        <v>68447694.868499994</v>
       </c>
       <c r="F7" s="14">
-        <f>F4*Assumptions!E5</f>
-        <v>338303.59253568004</v>
+        <f>E7*(1+Assumptions!E8)</f>
+        <v>78714849.098774984</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B8" s="14">
-        <f>Historicals!E10</f>
-        <v>38037063</v>
+        <f>Historicals!E11</f>
+        <v>37505395</v>
       </c>
       <c r="C8" s="14">
-        <f>B8*(1+Assumptions!B8)</f>
-        <v>47546328.75</v>
+        <f>B8*(1+Assumptions!B9)</f>
+        <v>48757013.5</v>
       </c>
       <c r="D8" s="14">
-        <f>C8*(1+Assumptions!C8)</f>
-        <v>58006521.074999996</v>
+        <f>C8*(1+Assumptions!C9)</f>
+        <v>60946266.875</v>
       </c>
       <c r="E8" s="14">
-        <f>D8*(1+Assumptions!D8)</f>
-        <v>68447694.868499994</v>
+        <f>D8*(1+Assumptions!D9)</f>
+        <v>73135520.25</v>
       </c>
       <c r="F8" s="14">
-        <f>E8*(1+Assumptions!E8)</f>
-        <v>78714849.098774984</v>
+        <f>E8*(1+Assumptions!E9)</f>
+        <v>86299913.894999996</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9" s="14">
-        <f>Historicals!E11</f>
-        <v>37505395</v>
+        <f>Historicals!E12</f>
+        <v>30319</v>
       </c>
       <c r="C9" s="14">
-        <f>B9*(1+Assumptions!B9)</f>
-        <v>48757013.5</v>
+        <f>C7*Assumptions!B10</f>
+        <v>38037.063000000002</v>
       </c>
       <c r="D9" s="14">
-        <f>C9*(1+Assumptions!C9)</f>
-        <v>60946266.875</v>
+        <f>D7*Assumptions!C10</f>
+        <v>46405.21686</v>
       </c>
       <c r="E9" s="14">
-        <f>D9*(1+Assumptions!D9)</f>
-        <v>73135520.25</v>
+        <f>E7*Assumptions!D10</f>
+        <v>61602.925381649991</v>
       </c>
       <c r="F9" s="14">
-        <f>E9*(1+Assumptions!E9)</f>
-        <v>86299913.894999996</v>
+        <f>F7*Assumptions!E10</f>
+        <v>78714.849098774983</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="14">
-        <f>Historicals!E12</f>
-        <v>30319</v>
-      </c>
-      <c r="C10" s="14">
-        <f>C8*Assumptions!B10</f>
-        <v>38037.063000000002</v>
-      </c>
-      <c r="D10" s="14">
-        <f>D8*Assumptions!C10</f>
-        <v>46405.21686</v>
-      </c>
-      <c r="E10" s="14">
-        <f>E8*Assumptions!D10</f>
-        <v>61602.925381649991</v>
-      </c>
-      <c r="F10" s="14">
-        <f>F8*Assumptions!E10</f>
-        <v>78714.849098774983</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="15">
+      <c r="B10" s="15">
         <f>Historicals!E6</f>
         <v>234151</v>
       </c>
-      <c r="C11" s="15">
-        <f>C4*Assumptions!B6</f>
+      <c r="C10" s="15">
+        <f>C3*Assumptions!B6</f>
         <v>260161.48799999998</v>
       </c>
-      <c r="D11" s="15">
-        <f>D4*Assumptions!C6</f>
+      <c r="D10" s="15">
+        <f>D3*Assumptions!C6</f>
         <v>296757.537312</v>
       </c>
-      <c r="E11" s="15">
-        <f>E4*Assumptions!D6</f>
+      <c r="E10" s="15">
+        <f>E3*Assumptions!D6</f>
         <v>326433.29104319995</v>
       </c>
-      <c r="F11" s="15">
-        <f>F4*Assumptions!E6</f>
+      <c r="F10" s="15">
+        <f>F3*Assumptions!E6</f>
         <v>372133.95178924804</v>
       </c>
     </row>
@@ -1935,19 +1929,19 @@
         <v>9</v>
       </c>
       <c r="B3" s="15">
-        <f>Forecast!C4</f>
+        <f>Forecast!C3</f>
         <v>4336024.8</v>
       </c>
       <c r="C3" s="15">
-        <f>Forecast!D4</f>
+        <f>Forecast!D3</f>
         <v>5116509.2639999995</v>
       </c>
       <c r="D3" s="15">
-        <f>Forecast!E4</f>
+        <f>Forecast!E3</f>
         <v>5935150.7462399993</v>
       </c>
       <c r="E3" s="15">
-        <f>Forecast!F4</f>
+        <f>Forecast!F3</f>
         <v>6766071.8507136004</v>
       </c>
     </row>
@@ -1956,19 +1950,19 @@
         <v>20</v>
       </c>
       <c r="B4" s="15">
-        <f>Forecast!C5</f>
+        <f>Forecast!C4</f>
         <v>1344167.6879999998</v>
       </c>
       <c r="C4" s="15">
-        <f>Forecast!D5</f>
+        <f>Forecast!D4</f>
         <v>1637282.9644799998</v>
       </c>
       <c r="D4" s="15">
-        <f>Forecast!E5</f>
+        <f>Forecast!E4</f>
         <v>1958599.7462591999</v>
       </c>
       <c r="E4" s="15">
-        <f>Forecast!F5</f>
+        <f>Forecast!F4</f>
         <v>2300464.4292426244</v>
       </c>
     </row>
@@ -1977,19 +1971,19 @@
         <v>11</v>
       </c>
       <c r="B5" s="15">
-        <f>Forecast!C11</f>
+        <f>Forecast!C10</f>
         <v>260161.48799999998</v>
       </c>
       <c r="C5" s="15">
-        <f>Forecast!D11</f>
+        <f>Forecast!D10</f>
         <v>296757.537312</v>
       </c>
       <c r="D5" s="15">
-        <f>Forecast!E11</f>
+        <f>Forecast!E10</f>
         <v>326433.29104319995</v>
       </c>
       <c r="E5" s="15">
-        <f>Forecast!F11</f>
+        <f>Forecast!F10</f>
         <v>372133.95178924804</v>
       </c>
     </row>
@@ -2082,19 +2076,19 @@
         <v>38</v>
       </c>
       <c r="B10" s="15">
-        <f>Forecast!C7</f>
+        <f>Forecast!C6</f>
         <v>216801.24</v>
       </c>
       <c r="C10" s="15">
-        <f>Forecast!D7</f>
+        <f>Forecast!D6</f>
         <v>255825.4632</v>
       </c>
       <c r="D10" s="15">
-        <f>Forecast!E7</f>
+        <f>Forecast!E6</f>
         <v>296757.537312</v>
       </c>
       <c r="E10" s="15">
-        <f>Forecast!F7</f>
+        <f>Forecast!F6</f>
         <v>338303.59253568004</v>
       </c>
     </row>
@@ -2300,7 +2294,7 @@
       </c>
     </row>
     <row r="37" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B37" s="42">
+      <c r="B37" s="41">
         <f>B24</f>
         <v>18.665387851754598</v>
       </c>
@@ -2691,7 +2685,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" s="41" t="s">
+      <c r="A30" t="s">
         <v>72</v>
       </c>
     </row>

</xml_diff>